<commit_message>
adding image to tab and adding download button for .ics file
</commit_message>
<xml_diff>
--- a/App_Data/AcademicCalendar.xlsx
+++ b/App_Data/AcademicCalendar.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\elie.tawk\source\repos\AcademicCalendarProject\App_Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{230D7B39-5FC2-4938-9BF7-276D25A1150E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37490C6E-1846-4825-B26F-44E345BA443C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{322C08C7-D37A-4DFC-8F83-221E70B99113}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$K$235</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$K$232</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1189" uniqueCount="453">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1169" uniqueCount="440">
   <si>
     <t>EventTitle</t>
   </si>
@@ -1356,49 +1356,10 @@
     <t>EVT-0231</t>
   </si>
   <si>
-    <t>Reminder Elie Test 1</t>
-  </si>
-  <si>
-    <t>Reminder Test Elie 1</t>
-  </si>
-  <si>
     <t>EVT-0232</t>
   </si>
   <si>
-    <t>Reminder Elie Test 2</t>
-  </si>
-  <si>
-    <t>Reminder Test Elie 2</t>
-  </si>
-  <si>
-    <t>EVT-0233</t>
-  </si>
-  <si>
-    <t>Reminder Elie Test 3</t>
-  </si>
-  <si>
-    <t>EVT-0234</t>
-  </si>
-  <si>
-    <t>Reminder Test Elie 3</t>
-  </si>
-  <si>
-    <t>Reminder Elie Test 4</t>
-  </si>
-  <si>
-    <t>Reminder Elie Test 5</t>
-  </si>
-  <si>
-    <t>Reminder Test Elie 4</t>
-  </si>
-  <si>
-    <t>Reminder Test Elie 5</t>
-  </si>
-  <si>
-    <t>EVT-0235</t>
-  </si>
-  <si>
-    <t>EVT-0236</t>
+    <t>Reminder Event 1</t>
   </si>
 </sst>
 </file>
@@ -1811,7 +1772,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{09AA4836-D25F-46B6-87A4-EE8D12FA65BD}">
-  <dimension ref="A1:K237"/>
+  <dimension ref="A1:K233"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="141.5546875" bestFit="1" customWidth="1"/>
@@ -7711,171 +7672,40 @@
     </row>
     <row r="233" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A233" s="4" t="s">
-        <v>438</v>
+        <v>26</v>
       </c>
       <c r="B233" s="4" t="s">
         <v>439</v>
       </c>
       <c r="C233" s="5">
-        <v>46273</v>
-      </c>
-      <c r="D233" s="6">
-        <v>0.875</v>
+        <v>46276</v>
+      </c>
+      <c r="D233" s="13">
+        <v>0.4236111111111111</v>
       </c>
       <c r="E233" s="5">
-        <v>46273</v>
+        <v>46276</v>
       </c>
       <c r="F233" s="6">
-        <v>0.95833333333333337</v>
-      </c>
-      <c r="G233" s="7"/>
+        <v>0.5</v>
+      </c>
       <c r="H233" s="4" t="s">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="I233" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="J233" s="4">
-        <v>5</v>
+      <c r="J233">
+        <v>2</v>
       </c>
       <c r="K233" s="8" t="s">
-        <v>440</v>
-      </c>
-    </row>
-    <row r="234" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A234" s="4" t="s">
-        <v>441</v>
-      </c>
-      <c r="B234" s="4" t="s">
-        <v>442</v>
-      </c>
-      <c r="C234" s="5">
-        <v>46276</v>
-      </c>
-      <c r="D234" s="6">
-        <v>0.34375</v>
-      </c>
-      <c r="E234" s="5">
-        <v>46276</v>
-      </c>
-      <c r="F234" s="6">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="G234" s="7"/>
-      <c r="H234" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="I234" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="J234" s="4">
-        <v>5</v>
-      </c>
-      <c r="K234" s="8" t="s">
-        <v>443</v>
-      </c>
-    </row>
-    <row r="235" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A235" s="4" t="s">
-        <v>444</v>
-      </c>
-      <c r="B235" s="4" t="s">
-        <v>446</v>
-      </c>
-      <c r="C235" s="5">
-        <v>46276</v>
-      </c>
-      <c r="D235" s="6">
-        <v>0.34375</v>
-      </c>
-      <c r="E235" s="5">
-        <v>46276</v>
-      </c>
-      <c r="F235" s="6">
-        <v>0.45833333333333331</v>
-      </c>
-      <c r="G235" s="7"/>
-      <c r="H235" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="I235" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="J235" s="4">
-        <v>5</v>
-      </c>
-      <c r="K235" s="8" t="s">
-        <v>445</v>
-      </c>
-    </row>
-    <row r="236" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A236" s="4" t="s">
-        <v>447</v>
-      </c>
-      <c r="B236" s="4" t="s">
-        <v>449</v>
-      </c>
-      <c r="C236" s="5">
-        <v>46277</v>
-      </c>
-      <c r="D236" s="13">
-        <v>0.375</v>
-      </c>
-      <c r="E236" s="5">
-        <v>46277</v>
-      </c>
-      <c r="F236" s="13">
-        <v>0.5</v>
-      </c>
-      <c r="H236" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="I236" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="J236">
-        <v>10</v>
-      </c>
-      <c r="K236" s="8" t="s">
-        <v>451</v>
-      </c>
-    </row>
-    <row r="237" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A237" s="4" t="s">
-        <v>448</v>
-      </c>
-      <c r="B237" s="4" t="s">
-        <v>450</v>
-      </c>
-      <c r="C237" s="5">
-        <v>46278</v>
-      </c>
-      <c r="D237" s="13">
-        <v>0.39583333333333331</v>
-      </c>
-      <c r="E237" s="5">
-        <v>46278</v>
-      </c>
-      <c r="F237" s="13">
-        <v>0.54166666666666663</v>
-      </c>
-      <c r="H237" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="I237" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="J237" s="4">
-        <v>15</v>
-      </c>
-      <c r="K237" s="8" t="s">
-        <v>452</v>
+        <v>438</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <dataValidations count="3">
-    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showDropDown="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid ReminderMinutes" error="ReminderMinutes must be a whole number greater than or equal to 0." promptTitle="ReminderMinutes" prompt="Optional. Enter minutes before event. Examples: 5, 15, 30, 60, 1440." sqref="J2:J235" xr:uid="{30CE5E6D-9715-456C-9318-D38C8910D564}">
+    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showDropDown="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid ReminderMinutes" error="ReminderMinutes must be a whole number greater than or equal to 0." promptTitle="ReminderMinutes" prompt="Optional. Enter minutes before event. Examples: 5, 15, 30, 60, 1440." sqref="J2:J232" xr:uid="{30CE5E6D-9715-456C-9318-D38C8910D564}">
       <formula1>0</formula1>
     </dataValidation>
     <dataValidation type="list" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid IsActive Value" error="Only Yes or No is allowed." promptTitle="IsActive" prompt="Select Yes or No." sqref="I1:I1048576" xr:uid="{B3E26B20-94DB-4F75-8C08-EBCD6153D2EB}">

</xml_diff>